<commit_message>
fix: align practice workbook with lessons and remove leaked answers
- Add Summary, E-Commerce and Warehouse sheets the lessons already
  referenced; Warehouse gains a stock = reorder point edge case
- Hide answers on the Warehouse capstone slide and fix slide 48/49
  subtitles to match the tasks
- Teach MAXIFS before SD-09; SD-10 now expects the FILTER spill
  instead of an untaught JOIN
- RG-07 expects "Bob Bob" without the trailing space; HR-01 names
  its source sheet
- Fix generator only updating answer_key.gs on the first run, and
  fail loudly if the answers block is missing
- Verify the new sheets, their expected results and SD-10 spill room

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Google_Sheets_Mastery_Practice.xlsx
+++ b/public/Google_Sheets_Mastery_Practice.xlsx
@@ -6,17 +6,20 @@
   <sheets>
     <sheet sheetId="1" name="Start_Here" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Classroom" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="HR_Roster" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Sales_Data" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Regex_Data" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Assignments" state="visible" r:id="rId9"/>
+    <sheet sheetId="3" name="Summary" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="HR_Roster" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Sales_Data" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Regex_Data" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Assignments" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="E-Commerce" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Warehouse" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="233">
   <si>
     <t>เริ่มเรียน</t>
   </si>
@@ -45,7 +48,7 @@
     <t>ตำแหน่งข้อมูล</t>
   </si>
   <si>
-    <t>HR_Roster / Sales_Data / Regex_Data: หัวตารางแถว 4 ข้อมูลเริ่มแถว 5</t>
+    <t>HR_Roster / Sales_Data / Regex_Data: หัวตารางแถว 4 ข้อมูลเริ่มแถว 5; Classroom / Summary / E-Commerce / Warehouse: หัวตารางแถว 1 ข้อมูลเริ่มแถว 2</t>
   </si>
   <si>
     <t>ช่องให้กรอก</t>
@@ -69,7 +72,19 @@
     <t>Classroom</t>
   </si>
   <si>
-    <t>ข้อมูลร้านค้าห้องเรียน: หัวแถว 1 ข้อมูลแถว 2–5; เติมสูตรใน E2:E5 และผลสรุปใน G2 เป็นต้นไป</t>
+    <t>ข้อมูลร้านค้าห้องเรียน: เติมสูตร Amount ใน E2:E5 และฝึก SUMIF ที่ G2 (กิจกรรมพื้นฐาน)</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>ตารางสรุปยอดแยกหมวดสำหรับทำกราฟและชิ้นงานพื้นฐาน: เติมสูตรในช่องสีเขียว B2:B3</t>
+  </si>
+  <si>
+    <t>ชิ้นงานต่อยอด</t>
+  </si>
+  <si>
+    <t>E-Commerce: เติม Net_Sales ใน G2:G4 แล้วสรุปด้วย QUERY; Warehouse: เติม SKU ใน E2:E4 และ Need_Restock ใน F2:F4</t>
   </si>
   <si>
     <t>วันที่</t>
@@ -81,7 +96,13 @@
     <t>Regex</t>
   </si>
   <si>
-    <t>ผลการสกัดมักเป็นข้อความ; RG-07 มีช่องว่างท้ายหนึ่งตัว; RG-08 คืนข้อความเต็มที่ปิด 4 หลักท้าย</t>
+    <t>ผลการสกัดมักเป็นข้อความ; RG-08 คืนข้อความเต็มที่ปิด 4 หลักท้าย</t>
+  </si>
+  <si>
+    <t>FILTER</t>
+  </si>
+  <si>
+    <t>SD-10 คืนผลหลายแถว (spill) ลงช่องด้านล่าง; เว้นช่องว่างใต้คำตอบไว้ ไม่เช่นนั้นจะเกิด #REF!</t>
   </si>
   <si>
     <t>ส่งงาน</t>
@@ -360,7 +381,7 @@
     <t>HR_Roster</t>
   </si>
   <si>
-    <t>นับจำนวนพนักงานทั้งหมดที่มีอยู่ในชีตนี้ (ใช้ COUNTA)</t>
+    <t>นับจำนวนพนักงานทั้งหมดในชีต HR_Roster (ใช้ COUNTA)</t>
   </si>
   <si>
     <t>7</t>
@@ -528,7 +549,7 @@
     <t>ดึงข้อมูล TransactionID ทั้งหมดของรายการที่มียอดขาย &gt; 100,000 บาท (ใช้ FILTER)</t>
   </si>
   <si>
-    <t>TX-1001, TX-1005</t>
+    <t>TX-1001 และ TX-1005 (แสดง 2 แถว)</t>
   </si>
   <si>
     <t>RG-01</t>
@@ -582,10 +603,10 @@
     <t>RG-07</t>
   </si>
   <si>
-    <t>ดึงชื่อคน (คำแรกสุดก่อนขีด -) ออกจาก Raw_Contact_Info ของ "R-003" (ใช้ REGEXEXTRACT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bob Bob </t>
+    <t>ดึงชื่อคน (ข้อความก่อนขีด - โดยไม่มีช่องว่างท้าย) ออกจาก Raw_Contact_Info ของ "R-003" (ใช้ REGEXEXTRACT)</t>
+  </si>
+  <si>
+    <t>Bob Bob</t>
   </si>
   <si>
     <t>RG-08</t>
@@ -613,6 +634,90 @@
   </si>
   <si>
     <t>TH2024_A12</t>
+  </si>
+  <si>
+    <t>TxnID</t>
+  </si>
+  <si>
+    <t>CustID</t>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <t>Gross_Sales</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>Is_Returned</t>
+  </si>
+  <si>
+    <t>Net_Sales</t>
+  </si>
+  <si>
+    <t>TX-901</t>
+  </si>
+  <si>
+    <t>CUST-551</t>
+  </si>
+  <si>
+    <t>Shopee</t>
+  </si>
+  <si>
+    <t>TX-902</t>
+  </si>
+  <si>
+    <t>CUST-882</t>
+  </si>
+  <si>
+    <t>Lazada</t>
+  </si>
+  <si>
+    <t>TX-903</t>
+  </si>
+  <si>
+    <t>CUST-104</t>
+  </si>
+  <si>
+    <t>TikTok</t>
+  </si>
+  <si>
+    <t>Bin_Location</t>
+  </si>
+  <si>
+    <t>Raw_Barcode</t>
+  </si>
+  <si>
+    <t>Unit_Stock</t>
+  </si>
+  <si>
+    <t>Reorder_Point</t>
+  </si>
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>Need_Restock</t>
+  </si>
+  <si>
+    <t>ZONE-A-01</t>
+  </si>
+  <si>
+    <t>[SKU-8821]-LOT4</t>
+  </si>
+  <si>
+    <t>ZONE-B-04</t>
+  </si>
+  <si>
+    <t>[SKU-9042]-LOT1</t>
+  </si>
+  <si>
+    <t>ZONE-C-02</t>
+  </si>
+  <si>
+    <t>[SKU-7730]-LOT2</t>
   </si>
 </sst>
 </file>
@@ -1118,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1219,6 +1324,30 @@
       </c>
       <c r="B12" s="1" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1241,27 +1370,27 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C2" s="3">
         <v>10</v>
@@ -1270,15 +1399,15 @@
         <v>20</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C3" s="3">
         <v>5</v>
@@ -1287,15 +1416,15 @@
         <v>10</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C4" s="3">
         <v>8</v>
@@ -1304,15 +1433,15 @@
         <v>7</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C5" s="3">
         <v>6</v>
@@ -1321,7 +1450,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1331,6 +1460,45 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1345,7 +1513,7 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1355,7 +1523,7 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1366,33 +1534,33 @@
     <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D5" s="13">
         <v>44576</v>
@@ -1406,13 +1574,13 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D6" s="13">
         <v>45444</v>
@@ -1426,13 +1594,13 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D7" s="13">
         <v>45981</v>
@@ -1446,13 +1614,13 @@
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D8" s="13">
         <v>44265</v>
@@ -1466,13 +1634,13 @@
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D9" s="13">
         <v>46054</v>
@@ -1486,13 +1654,13 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>58</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>52</v>
       </c>
       <c r="D10" s="13">
         <v>44058</v>
@@ -1506,13 +1674,13 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D11" s="13">
         <v>45170</v>
@@ -1534,7 +1702,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1548,7 +1716,7 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1558,7 +1726,7 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1569,33 +1737,33 @@
     <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D5" s="13">
         <v>46285</v>
@@ -1609,13 +1777,13 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D6" s="13">
         <v>46285</v>
@@ -1629,13 +1797,13 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D7" s="13">
         <v>46286</v>
@@ -1649,13 +1817,13 @@
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D8" s="13">
         <v>46286</v>
@@ -1669,13 +1837,13 @@
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D9" s="13">
         <v>46287</v>
@@ -1689,13 +1857,13 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D10" s="13">
         <v>46287</v>
@@ -1709,13 +1877,13 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>80</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>74</v>
       </c>
       <c r="D11" s="13">
         <v>46288</v>
@@ -1737,7 +1905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1749,7 +1917,7 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1757,7 +1925,7 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1766,86 +1934,86 @@
     <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1858,7 +2026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1872,7 +2040,7 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1881,7 +2049,7 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1891,563 +2059,563 @@
     <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>113</v>
-      </c>
       <c r="C7" s="12" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>143</v>
-      </c>
       <c r="C18" s="12" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="E22" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E25" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E27" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="B30" s="12" t="s">
-        <v>172</v>
-      </c>
       <c r="C30" s="12" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="E31" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E35" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2458,4 +2626,212 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="7" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2450</v>
+      </c>
+      <c r="E2" s="3">
+        <v>250</v>
+      </c>
+      <c r="F2" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D3" s="3">
+        <v>8900</v>
+      </c>
+      <c r="E3" s="3">
+        <v>500</v>
+      </c>
+      <c r="F3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="3">
+        <v>140</v>
+      </c>
+      <c r="D2" s="3">
+        <v>50</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C3" s="3">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3">
+        <v>30</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C4" s="3">
+        <v>25</v>
+      </c>
+      <c r="D4" s="3">
+        <v>25</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add self-check column and score to practice assignments
Assignments!F shows ✓/✗ as learners type, flags typed values that
are not formulas, and F3 totals the score out of 30. The check
formulas come from scripts/self-check.cjs, shared with the verifier,
which rebuilds each one from values computed from the data.

Also write learner and separator cells as truly empty instead of
empty strings, which blocked the SD-10 FILTER spill.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Google_Sheets_Mastery_Practice.xlsx
+++ b/public/Google_Sheets_Mastery_Practice.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="234">
   <si>
     <t>เริ่มเรียน</t>
   </si>
@@ -66,7 +66,7 @@
     <t>ตรวจคำตอบ</t>
   </si>
   <si>
-    <t>เทียบผลกับคอลัมน์ D; เฉลยพร้อมเหตุผลอยู่หน้าเฉลยในเว็บ เปิดดูทีละข้อหลังลองทำ</t>
+    <t>คอลัมน์ F (Self_Check) ขึ้น ✓ เมื่อผลถูก ✗ เมื่อยังไม่ตรง และ ⚠ ถ้าพิมพ์ค่าแทนสูตร คะแนนรวมอยู่ที่ F3; เฉลยพร้อมเหตุผลอยู่หน้าเฉลยในเว็บ</t>
   </si>
   <si>
     <t>Classroom</t>
@@ -132,9 +132,6 @@
     <t>เครื่องเขียน</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>ดินสอ</t>
   </si>
   <si>
@@ -357,7 +354,10 @@
     <t>TH2025-B44</t>
   </si>
   <si>
-    <t>บททดสอบท้ายบทเรียน (รวม 30 ข้อ) ให้นำความรู้ทั้งหมดมาแก้ไขโจทย์ด้านล่าง โดยให้ผู้เรียนพิมพ์สูตรเพื่อหาคำตอบลงในคอลัมน์ Your_Formula สีเขียว ให้ตรงกับ Expected Result</t>
+    <t>บททดสอบท้ายบทเรียน (รวม 30 ข้อ) พิมพ์สูตรในคอลัมน์ Your_Formula สีเขียว คอลัมน์ Self_Check จะบอกทันทีว่าผลตรงกับ Expected_Result หรือไม่ และเตือนถ้าพิมพ์ตัวเลขแทนสูตร</t>
+  </si>
+  <si>
+    <t>คะแนนตรวจตัวเอง</t>
   </si>
   <si>
     <t>Task_ID</t>
@@ -373,6 +373,9 @@
   </si>
   <si>
     <t>Your_Formula</t>
+  </si>
+  <si>
+    <t>Self_Check</t>
   </si>
   <si>
     <t>HR-01</t>
@@ -728,7 +731,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;฿&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -760,6 +763,12 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="18"/>
+      <name val="TH Sarabun New"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF059669"/>
+      <sz val="16"/>
       <name val="TH Sarabun New"/>
     </font>
   </fonts>
@@ -833,7 +842,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -881,14 +890,57 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF047857"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFB91C1C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFB45309"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1398,13 +1450,11 @@
       <c r="D2" s="3">
         <v>20</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="E2" s="4"/>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>36</v>
@@ -1415,16 +1465,14 @@
       <c r="D3" s="3">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="C4" s="3">
         <v>8</v>
@@ -1432,16 +1480,14 @@
       <c r="D4" s="3">
         <v>7</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="E4" s="4"/>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" s="3">
         <v>6</v>
@@ -1449,9 +1495,7 @@
       <c r="D5" s="3">
         <v>15</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="E5" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1480,17 +1524,13 @@
       <c r="A2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="B2" s="4"/>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>37</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B3" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1513,7 +1553,7 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1523,7 +1563,7 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1534,33 +1574,33 @@
     <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="F4" s="9" t="s">
         <v>48</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="12" t="s">
         <v>51</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>52</v>
       </c>
       <c r="D5" s="13">
         <v>44576</v>
@@ -1574,13 +1614,13 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" s="12" t="s">
         <v>54</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>55</v>
       </c>
       <c r="D6" s="13">
         <v>45444</v>
@@ -1594,13 +1634,13 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="12" t="s">
         <v>57</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>58</v>
       </c>
       <c r="D7" s="13">
         <v>45981</v>
@@ -1614,13 +1654,13 @@
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>60</v>
-      </c>
       <c r="C8" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D8" s="13">
         <v>44265</v>
@@ -1634,13 +1674,13 @@
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="D9" s="13">
         <v>46054</v>
@@ -1654,13 +1694,13 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>65</v>
-      </c>
       <c r="C10" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D10" s="13">
         <v>44058</v>
@@ -1674,13 +1714,13 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="12" t="s">
-        <v>67</v>
-      </c>
       <c r="C11" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D11" s="13">
         <v>45170</v>
@@ -1716,7 +1756,7 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1726,7 +1766,7 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1737,33 +1777,33 @@
     <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="F4" s="18" t="s">
         <v>73</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>77</v>
       </c>
       <c r="D5" s="13">
         <v>46285</v>
@@ -1777,13 +1817,13 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" s="12" t="s">
         <v>79</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>80</v>
       </c>
       <c r="D6" s="13">
         <v>46285</v>
@@ -1797,13 +1837,13 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>82</v>
-      </c>
       <c r="C7" s="12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D7" s="13">
         <v>46286</v>
@@ -1817,13 +1857,13 @@
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D8" s="13">
         <v>46286</v>
@@ -1837,13 +1877,13 @@
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" s="13">
         <v>46287</v>
@@ -1857,13 +1897,13 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B10" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>77</v>
       </c>
       <c r="D10" s="13">
         <v>46287</v>
@@ -1877,13 +1917,13 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D11" s="13">
         <v>46288</v>
@@ -1917,7 +1957,7 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1925,7 +1965,7 @@
     </row>
     <row r="2" ht="35" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1934,86 +1974,86 @@
     <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>90</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="12" t="s">
         <v>94</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="D6" s="12" t="s">
         <v>98</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="D7" s="12" t="s">
         <v>102</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="C8" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="D8" s="12" t="s">
         <v>106</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="D9" s="12" t="s">
         <v>110</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2028,7 +2068,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2036,28 +2076,38 @@
     <col min="3" max="3" width="75" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
       <c r="E1" s="7"/>
-    </row>
-    <row r="2" ht="35" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="7"/>
+    </row>
+    <row r="2" ht="35" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
-    </row>
-    <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="8"/>
+    </row>
+    <row r="3" ht="26" customHeight="1" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E3" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" s="22">
+        <f>COUNTIF(F5:F36,"✓ ถูกต้อง")&amp;" / 30"</f>
+      </c>
+    </row>
+    <row r="4" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>113</v>
       </c>
@@ -2073,556 +2123,568 @@
       <c r="E4" s="9" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="23"/>
+      <c r="F5" s="24">
+        <f>IF(E5="","",IF(NOT(ISFORMULA(E5)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E5,2)=7,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>119</v>
-      </c>
       <c r="C6" s="12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+      <c r="E6" s="23"/>
+      <c r="F6" s="24">
+        <f>IF(E6="","",IF(NOT(ISFORMULA(E6)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E6,2)=2,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E7" s="23"/>
+      <c r="F7" s="24">
+        <f>IF(E7="","",IF(NOT(ISFORMULA(E7)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E7,2)=2,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="E8" s="23"/>
+      <c r="F8" s="24">
+        <f>IF(E8="","",IF(NOT(ISFORMULA(E8)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E8,2)=358000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="E9" s="23"/>
+      <c r="F9" s="24">
+        <f>IF(E9="","",IF(NOT(ISFORMULA(E9)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E9,2)=86000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+      <c r="E10" s="23"/>
+      <c r="F10" s="24">
+        <f>IF(E10="","",IF(NOT(ISFORMULA(E10)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E10,2)=50000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="E11" s="23"/>
+      <c r="F11" s="24">
+        <f>IF(E11="","",IF(NOT(ISFORMULA(E11)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E11,2)=85000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E12" s="23"/>
+      <c r="F12" s="24">
+        <f>IF(E12="","",IF(NOT(ISFORMULA(E12)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(E12=DATEDIF(HR_Roster!D8,TODAY(),"Y"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="E13" s="23"/>
+      <c r="F13" s="24">
+        <f>IF(E13="","",IF(NOT(ISFORMULA(E13)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(E13=TRUE,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="E14" s="23"/>
+      <c r="F14" s="24">
+        <f>IF(E14="","",IF(NOT(ISFORMULA(E14)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E14,"Business"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E16" s="23"/>
+      <c r="F16" s="24">
+        <f>IF(E16="","",IF(NOT(ISFORMULA(E16)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E16,2)=593000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="E17" s="23"/>
+      <c r="F17" s="24">
+        <f>IF(E17="","",IF(NOT(ISFORMULA(E17)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E17,2)=198000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="E18" s="23"/>
+      <c r="F18" s="24">
+        <f>IF(E18="","",IF(NOT(ISFORMULA(E18)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E18,2)=310000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="E19" s="23"/>
+      <c r="F19" s="24">
+        <f>IF(E19="","",IF(NOT(ISFORMULA(E19)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E19,2)=2,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="E20" s="23"/>
+      <c r="F20" s="24">
+        <f>IF(E20="","",IF(NOT(ISFORMULA(E20)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E20,2)=180,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="E21" s="23"/>
+      <c r="F21" s="24">
+        <f>IF(E21="","",IF(NOT(ISFORMULA(E21)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E21,2)=30000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E22" s="23"/>
+      <c r="F22" s="24">
+        <f>IF(E22="","",IF(NOT(ISFORMULA(E22)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E22,"Office Supplies"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="E23" s="23"/>
+      <c r="F23" s="24">
+        <f>IF(E23="","",IF(NOT(ISFORMULA(E23)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E23,2)=1,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="23"/>
+      <c r="F24" s="24">
+        <f>IF(E24="","",IF(NOT(ISFORMULA(E24)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(ROUND(E24,2)=125000,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="E25" s="23"/>
+      <c r="F25" s="24">
+        <f>IF(E25="","",IF(NOT(ISFORMULA(E25)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(OR(AND(E25="TX-1001",E26="TX-1005"),E25="TX-1001, TX-1005"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D27" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="B14" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="E21" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="E22" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>173</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="C27" s="12" t="s">
+      <c r="E27" s="23"/>
+      <c r="F27" s="24">
+        <f>IF(E27="","",IF(NOT(ISFORMULA(E27)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(E27=TRUE,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="D27" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>178</v>
-      </c>
       <c r="C28" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="E28" s="23"/>
+      <c r="F28" s="24">
+        <f>IF(E28="","",IF(NOT(ISFORMULA(E28)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(E28=TRUE,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="E29" s="23"/>
+      <c r="F29" s="24">
+        <f>IF(E29="","",IF(NOT(ISFORMULA(E29)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(E29=TRUE,FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="E30" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+      <c r="E30" s="23"/>
+      <c r="F30" s="24">
+        <f>IF(E30="","",IF(NOT(ISFORMULA(E30)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E30,"yahoo.com"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+      <c r="E31" s="23"/>
+      <c r="F31" s="24">
+        <f>IF(E31="","",IF(NOT(ISFORMULA(E31)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E31,"450"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>192</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+      <c r="E32" s="23"/>
+      <c r="F32" s="24">
+        <f>IF(E32="","",IF(NOT(ISFORMULA(E32)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E32,"2025"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>195</v>
-      </c>
-      <c r="E33" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+      <c r="E33" s="23"/>
+      <c r="F33" s="24">
+        <f>IF(E33="","",IF(NOT(ISFORMULA(E33)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E33,"Bob Bob"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+      <c r="E34" s="23"/>
+      <c r="F34" s="24">
+        <f>IF(E34="","",IF(NOT(ISFORMULA(E34)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E34,"Alice - alice@company.co.th / 085999****"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="E35" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+      <c r="E35" s="23"/>
+      <c r="F35" s="24">
+        <f>IF(E35="","",IF(NOT(ISFORMULA(E35)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E35,"1200"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>37</v>
+        <v>205</v>
+      </c>
+      <c r="E36" s="23"/>
+      <c r="F36" s="24">
+        <f>IF(E36="","",IF(NOT(ISFORMULA(E36)),"⚠ พิมพ์เป็นสูตร",IF(IFERROR(EXACT(E36,"TH2024_A12"),FALSE),"✓ ถูกต้อง","✗ ยังไม่ตรง")))</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
   </mergeCells>
+  <conditionalFormatting sqref="F5:F36">
+    <cfRule type="containsText" dxfId="0" priority="1">
+      <formula>NOT(ISERROR(SEARCH("✓",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2">
+      <formula>NOT(ISERROR(SEARCH("✗",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3">
+      <formula>NOT(ISERROR(SEARCH("⚠",F5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2641,36 +2703,36 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D2" s="3">
         <v>2450</v>
@@ -2681,19 +2743,17 @@
       <c r="F2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D3" s="3">
         <v>8900</v>
@@ -2704,19 +2764,17 @@
       <c r="F3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D4" s="3">
         <v>1200</v>
@@ -2727,9 +2785,7 @@
       <c r="F4" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="G4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2752,30 +2808,30 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C2" s="3">
         <v>140</v>
@@ -2783,19 +2839,15 @@
       <c r="D2" s="3">
         <v>50</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C3" s="3">
         <v>12</v>
@@ -2803,19 +2855,15 @@
       <c r="D3" s="3">
         <v>30</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C4" s="3">
         <v>25</v>
@@ -2823,12 +2871,8 @@
       <c r="D4" s="3">
         <v>25</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>